<commit_message>
feat: melhorias de UI, dados e integracao de contratos 2026
Templates - Contratos Dashboard:
- Adiciona plugin ChartDataLabels ao grafico de contratos por status
- Exibe rotulo de valor diretamente nas barras (anchor end, clamp true)
- Melhora layout do grafico de execucao orcamentaria (grid oculto, eixo X ocultado)
- Desativa datalabels no grafico empilhado de execucao (tooltip suficiente)

Templates - Empenhos:
- Ajustes de layout e exibicao na tela de empenhos SIAFE

Templates - SRP Dashboard e Contratacoes Decorrentes:
- Refinamentos visuais na listagem de contratacoes decorrentes
- Melhorias no dashboard SRP (filtros, contagens, exibicao de status)

Dados - Planilha Oficial de Contratos 2026:
- Adiciona PAINEL DE CONTRATOS 2026(PAINEL).csv (planilha validada pela equipe de gestao)
- Adiciona PAINEL DE CONTRATOS 2026.xlsx (versao original)
- Atualiza ACOMPANHAMENTO-CONTRATOS 2026.xlsx com dados recentes
</commit_message>
<xml_diff>
--- a/data/contratos/ACOMPANHAMENTO-CONTRATOS 2026.xlsx
+++ b/data/contratos/ACOMPANHAMENTO-CONTRATOS 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30318"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01789F3A-0684-44FA-8688-9584331B951B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA4EC7E3-6F50-4F3F-B694-4802A4B99F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="253">
   <si>
     <t>CONTRATOS MP/PI- 2026</t>
   </si>
@@ -751,6 +751,164 @@
     <t>MAURO C O LOPES LTDA CNPJ/MF sob o nº 00.375.697/0001-85</t>
   </si>
   <si>
+    <t>35/2026</t>
+  </si>
+  <si>
+    <t>19.21.0785.0024228/2026-51</t>
+  </si>
+  <si>
+    <t>registro de preços, pelo prazo de 12 (doze) meses, para a contratação de postos para os serviços continuados de Auxiliar Administrativo, Agente de Limpeza, Auxiliar de Serviços Gerais, Bombeiro Hidráulico, Carregador de Volumes, Copeiragem, Eletricista, Garçonaria, Motorista Categoria A (motoboy), Motorista Categoria B (condução de veículo leve), Motorista Categoria D (condução de veículo pesado), Office Boy, Operador de Som e Imagem, Recepcionista, Recepcionista Bilíngue e Telefonista, a serem executados com regime de dedicação exclusiva de mão de obra, conforme condições e especificações estabelecidas no Termo de Referência</t>
+  </si>
+  <si>
+    <t>LOTE 1</t>
+  </si>
+  <si>
+    <t>ALFA GESTÃO DE RECURSOS HUMANOS LTDA, CNPJ: 07.204.255/0001-15</t>
+  </si>
+  <si>
+    <t>36/2026</t>
+  </si>
+  <si>
+    <t>19.21.0785.0023671/2026-55</t>
+  </si>
+  <si>
+    <t>contratação de 46 postos para os serviços continuados de Agente de Limpeza, a serem executados com regime de dedicação exclusiva de mão de obra</t>
+  </si>
+  <si>
+    <t>P.E Nº 90003/2026 Nº 11/2026</t>
+  </si>
+  <si>
+    <t>37/2026</t>
+  </si>
+  <si>
+    <t>19.21.0412.0011743/2026-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adesão à Ata de Registro de Preço n.º 114/2025 do Pregão Eletrônico n.º 057/2025 /SECRETARIA DAADMINISTRAÇÃO DO ESTADO DA BAHIA - SAEB, para aquisição de veículos automotores pick up </t>
+  </si>
+  <si>
+    <t>Adesão nº 02/2026</t>
+  </si>
+  <si>
+    <t>ARP Nº 114/2025,          P. E. Nº 057/2025</t>
+  </si>
+  <si>
+    <t>HPE AUTOMOTORES DO BRASIL LTDA, CNPJ: 54.305.743/0011-70</t>
+  </si>
+  <si>
+    <t>38/2026</t>
+  </si>
+  <si>
+    <t>19.21.0431.0022103/2026-74</t>
+  </si>
+  <si>
+    <t>contratação de empresa especializada na prestação de serviços de conservação e manutenção predial, com fornecimento e aplicação de materiais, destinados aos imóveis do Ministério Público do Estado do Piauí</t>
+  </si>
+  <si>
+    <t>P.E. Nº 90004/2026</t>
+  </si>
+  <si>
+    <t>ATA Nº 12/2026 </t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>19.21.0016.0026251/2026-33</t>
+  </si>
+  <si>
+    <t>quisição de suprimentos e ferramentas de TIC para atender as necessidades da Divisão de Atendimento ao Usuário, vinculada a Coordenadoria de Tecnologia da Informação do MPPI</t>
+  </si>
+  <si>
+    <r>
+      <t>Pregão Eletrônico nº </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cambria"/>
+        <charset val="1"/>
+      </rPr>
+      <t>90012/2026</t>
+    </r>
+  </si>
+  <si>
+    <t>ARP nº 15/2026</t>
+  </si>
+  <si>
+    <t>RRM SERVIÇOS E COMÉRCIOS DE CARTUCHOS LTDA</t>
+  </si>
+  <si>
+    <t>40/2026</t>
+  </si>
+  <si>
+    <t>19.21.0427.0026200/2026-95</t>
+  </si>
+  <si>
+    <t>aquisição de equipamentos de segurança eletrônica, vídeo monitoramento (CFTV),
+controle de acesso e alarmes</t>
+  </si>
+  <si>
+    <t>P.E. Nº  90016/2026</t>
+  </si>
+  <si>
+    <t>ATA Nº 19/2026</t>
+  </si>
+  <si>
+    <t>L F DE LIMA
+CNPJ: 48.614.060/0001-20</t>
+  </si>
+  <si>
+    <t>41/2026</t>
+  </si>
+  <si>
+    <t>19.21.0427.0026204/2026-84</t>
+  </si>
+  <si>
+    <t>ATA Nº 20/2026</t>
+  </si>
+  <si>
+    <t>LOTE III e IV</t>
+  </si>
+  <si>
+    <t>DOUBLE SOLUÇÕES E TECNOLOGIA
+CNPJ:26.587.509/0001-76</t>
+  </si>
+  <si>
+    <t>42/2026</t>
+  </si>
+  <si>
+    <t>19.21.0427.0026182/2026-96</t>
+  </si>
+  <si>
+    <t>Aquisição de equipamentos de segurança eletrônica, vídeo monitoramento (CFTV),
+controle de acesso e alarmes</t>
+  </si>
+  <si>
+    <t>L F COMÉRCIO DE ELETRÔNICOS LTDA, CNPJ: 52.585.078/0001-19</t>
+  </si>
+  <si>
+    <t>43/2026</t>
+  </si>
+  <si>
+    <t>19.21.0016.0026306/2026-03</t>
+  </si>
+  <si>
+    <t>Aquisição de Conectores RJ-45 EZ Crimp – CAT6 (pacote com 100), Alicate de crimpagem com catraca EZ Crimp e Cabo UTP CAT. 6 para suprir as necessidades da Divisão de Atendimento ao Usuário (Lote 3).</t>
+  </si>
+  <si>
+    <t>ATA Nº 17/2026 </t>
+  </si>
+  <si>
+    <t>DOMINI TELECOM LTDA |
+CNPJ: 46.869.912/0001-03</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
     <t>ATUALIZAÇÃO DO CABEÇALHO DOS CONTRATOS - Fundo e PGJ</t>
   </si>
   <si>
@@ -774,7 +932,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]General"/>
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -939,6 +1097,25 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Cambria"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1188,14 +1365,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1204,7 +1383,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1428,12 +1607,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1441,9 +1614,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1451,22 +1621,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1475,20 +1630,8 @@
     <xf numFmtId="14" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1499,9 +1642,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1511,25 +1651,96 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1854,7 +2065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M150"/>
+  <dimension ref="A1:M152"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.85546875" style="1" customWidth="1"/>
@@ -1874,62 +2085,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15" customHeight="1">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="129" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
+      <c r="L1" s="130"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1">
-      <c r="A2" s="116"/>
-      <c r="B2" s="117"/>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="117"/>
-      <c r="H2" s="117"/>
-      <c r="I2" s="117"/>
-      <c r="J2" s="117"/>
-      <c r="K2" s="117"/>
-      <c r="L2" s="117"/>
+      <c r="A2" s="129"/>
+      <c r="B2" s="130"/>
+      <c r="C2" s="130"/>
+      <c r="D2" s="130"/>
+      <c r="E2" s="130"/>
+      <c r="F2" s="130"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="130"/>
+      <c r="K2" s="130"/>
+      <c r="L2" s="130"/>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1">
-      <c r="A3" s="116"/>
-      <c r="B3" s="117"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="117"/>
-      <c r="F3" s="117"/>
-      <c r="G3" s="117"/>
-      <c r="H3" s="117"/>
-      <c r="I3" s="117"/>
-      <c r="J3" s="117"/>
-      <c r="K3" s="117"/>
-      <c r="L3" s="117"/>
+      <c r="A3" s="129"/>
+      <c r="B3" s="130"/>
+      <c r="C3" s="130"/>
+      <c r="D3" s="130"/>
+      <c r="E3" s="130"/>
+      <c r="F3" s="130"/>
+      <c r="G3" s="130"/>
+      <c r="H3" s="130"/>
+      <c r="I3" s="130"/>
+      <c r="J3" s="130"/>
+      <c r="K3" s="130"/>
+      <c r="L3" s="130"/>
     </row>
     <row r="4" spans="1:13" ht="22.5" customHeight="1">
-      <c r="A4" s="116"/>
-      <c r="B4" s="117"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
-      <c r="L4" s="117"/>
+      <c r="A4" s="129"/>
+      <c r="B4" s="130"/>
+      <c r="C4" s="130"/>
+      <c r="D4" s="130"/>
+      <c r="E4" s="130"/>
+      <c r="F4" s="130"/>
+      <c r="G4" s="130"/>
+      <c r="H4" s="130"/>
+      <c r="I4" s="130"/>
+      <c r="J4" s="130"/>
+      <c r="K4" s="130"/>
+      <c r="L4" s="130"/>
     </row>
     <row r="5" spans="1:13" ht="81" customHeight="1">
       <c r="A5" s="11" t="s">
@@ -2741,28 +2952,28 @@
       </c>
     </row>
     <row r="26" spans="1:13" ht="45.75">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="92" t="s">
         <v>122</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="84" t="s">
         <v>117</v>
       </c>
-      <c r="C26" s="89" t="s">
+      <c r="C26" s="115" t="s">
         <v>123</v>
       </c>
       <c r="D26" s="79" t="s">
         <v>124</v>
       </c>
-      <c r="E26" s="34" t="s">
+      <c r="E26" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="83" t="s">
         <v>125</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="83" t="s">
         <v>126</v>
       </c>
-      <c r="H26" s="78" t="s">
+      <c r="H26" s="116" t="s">
         <v>127</v>
       </c>
       <c r="I26" s="58">
@@ -2777,36 +2988,36 @@
       <c r="L26" s="58">
         <v>46106</v>
       </c>
-      <c r="M26" s="96">
+      <c r="M26" s="88">
         <v>46111</v>
       </c>
     </row>
     <row r="27" spans="1:13" s="24" customFormat="1" ht="30" customHeight="1">
-      <c r="A27" s="61" t="s">
+      <c r="A27" s="99" t="s">
         <v>128</v>
       </c>
-      <c r="B27" s="34" t="s">
+      <c r="B27" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="90" t="s">
+      <c r="C27" s="100" t="s">
         <v>129</v>
       </c>
-      <c r="D27" s="62" t="s">
+      <c r="D27" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="F27" s="62" t="s">
+      <c r="F27" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="G27" s="62" t="s">
+      <c r="G27" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="H27" s="62" t="s">
+      <c r="H27" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="I27" s="75">
+      <c r="I27" s="110">
         <v>45740</v>
       </c>
       <c r="J27" s="75">
@@ -2818,36 +3029,36 @@
       <c r="L27" s="75">
         <v>46107</v>
       </c>
-      <c r="M27" s="96">
+      <c r="M27" s="88">
         <v>46111</v>
       </c>
     </row>
     <row r="28" spans="1:13" s="24" customFormat="1" ht="57" customHeight="1">
-      <c r="A28" s="61" t="s">
+      <c r="A28" s="99" t="s">
         <v>134</v>
       </c>
-      <c r="B28" s="34" t="s">
+      <c r="B28" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="74" t="s">
+      <c r="C28" s="101" t="s">
         <v>135</v>
       </c>
-      <c r="D28" s="79" t="s">
+      <c r="D28" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="F28" s="62" t="s">
+      <c r="F28" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="G28" s="79" t="s">
+      <c r="G28" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="H28" s="62" t="s">
+      <c r="H28" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="I28" s="75">
+      <c r="I28" s="110">
         <v>45740</v>
       </c>
       <c r="J28" s="75">
@@ -2859,139 +3070,139 @@
       <c r="L28" s="75">
         <v>46107</v>
       </c>
-      <c r="M28" s="96">
+      <c r="M28" s="88">
         <v>46111</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="30">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="86" t="s">
+      <c r="C29" s="102" t="s">
         <v>141</v>
       </c>
       <c r="D29" s="80" t="s">
         <v>142</v>
       </c>
-      <c r="E29" s="87" t="s">
+      <c r="E29" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F29" s="81" t="s">
+      <c r="F29" s="103" t="s">
         <v>143</v>
       </c>
-      <c r="G29" s="86" t="s">
+      <c r="G29" s="102" t="s">
         <v>132</v>
       </c>
       <c r="H29" s="80" t="s">
         <v>144</v>
       </c>
-      <c r="I29" s="88"/>
-      <c r="J29" s="88"/>
-      <c r="K29" s="88"/>
-      <c r="L29" s="88"/>
-      <c r="M29" s="88"/>
+      <c r="I29" s="111"/>
+      <c r="J29" s="85"/>
+      <c r="K29" s="85"/>
+      <c r="L29" s="85"/>
+      <c r="M29" s="85"/>
     </row>
     <row r="30" spans="1:13" ht="60.75">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B30" s="85" t="s">
+      <c r="B30" s="18" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="D30" s="82" t="s">
+      <c r="D30" s="80" t="s">
         <v>147</v>
       </c>
       <c r="E30" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F30" s="83" t="s">
+      <c r="F30" s="81" t="s">
         <v>148</v>
       </c>
       <c r="G30" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="H30" s="82" t="s">
+      <c r="H30" s="80" t="s">
         <v>150</v>
       </c>
-      <c r="I30" s="84"/>
-      <c r="J30" s="84"/>
-      <c r="K30" s="84"/>
-      <c r="L30" s="84"/>
-      <c r="M30" s="84"/>
+      <c r="I30" s="112"/>
+      <c r="J30" s="82"/>
+      <c r="K30" s="82"/>
+      <c r="L30" s="82"/>
+      <c r="M30" s="82"/>
     </row>
     <row r="31" spans="1:13" s="24" customFormat="1" ht="45.75">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="99" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="62" t="s">
+      <c r="B31" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="97" t="s">
+      <c r="C31" s="101" t="s">
         <v>152</v>
       </c>
-      <c r="D31" s="91" t="s">
+      <c r="D31" s="21" t="s">
         <v>153</v>
       </c>
       <c r="E31" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F31" s="91" t="s">
+      <c r="F31" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="G31" s="94" t="s">
+      <c r="G31" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="H31" s="94" t="s">
+      <c r="H31" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="I31" s="98">
+      <c r="I31" s="113">
         <v>46111</v>
       </c>
-      <c r="J31" s="98">
+      <c r="J31" s="89">
         <v>46112</v>
       </c>
-      <c r="K31" s="98">
+      <c r="K31" s="89">
         <v>46111</v>
       </c>
-      <c r="L31" s="98">
+      <c r="L31" s="89">
         <v>46113</v>
       </c>
-      <c r="M31" s="98">
+      <c r="M31" s="89">
         <v>46113</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="66.75">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="C32" s="77" t="s">
+      <c r="C32" s="70" t="s">
         <v>158</v>
       </c>
-      <c r="D32" s="92" t="s">
+      <c r="D32" s="86" t="s">
         <v>159</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F32" s="92" t="s">
+      <c r="F32" s="86" t="s">
         <v>160</v>
       </c>
-      <c r="G32" s="95" t="s">
+      <c r="G32" s="87" t="s">
         <v>161</v>
       </c>
-      <c r="H32" s="93" t="s">
+      <c r="H32" s="86" t="s">
         <v>162</v>
       </c>
-      <c r="I32" s="110">
+      <c r="I32" s="96">
         <v>46120</v>
       </c>
       <c r="J32" s="76">
@@ -3006,31 +3217,31 @@
       <c r="M32" s="5"/>
     </row>
     <row r="33" spans="1:13" ht="45.75">
-      <c r="A33" s="104" t="s">
+      <c r="A33" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="B33" s="87" t="s">
+      <c r="B33" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="87" t="s">
+      <c r="C33" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D33" s="24" t="s">
+      <c r="D33" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="E33" s="86" t="s">
+      <c r="E33" s="102" t="s">
         <v>78</v>
       </c>
-      <c r="F33" s="99" t="s">
+      <c r="F33" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="G33" s="105" t="s">
+      <c r="G33" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H33" s="100" t="s">
+      <c r="H33" s="81" t="s">
         <v>167</v>
       </c>
-      <c r="I33" s="5"/>
+      <c r="I33" s="50"/>
       <c r="J33" s="5"/>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
@@ -3046,22 +3257,22 @@
       <c r="C34" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="D34" s="102" t="s">
+      <c r="D34" s="90" t="s">
         <v>170</v>
       </c>
       <c r="E34" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F34" s="103" t="s">
+      <c r="F34" s="91" t="s">
         <v>171</v>
       </c>
-      <c r="G34" s="108" t="s">
+      <c r="G34" s="95" t="s">
         <v>172</v>
       </c>
       <c r="H34" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="I34" s="110">
+      <c r="I34" s="96">
         <v>46128</v>
       </c>
       <c r="J34" s="5"/>
@@ -3070,118 +3281,118 @@
       <c r="M34" s="5"/>
     </row>
     <row r="35" spans="1:13" ht="61.5">
-      <c r="A35" s="106" t="s">
+      <c r="A35" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="B35" s="101" t="s">
+      <c r="B35" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C35" s="101" t="s">
+      <c r="C35" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="D35" s="109" t="s">
+      <c r="D35" s="97" t="s">
         <v>176</v>
       </c>
-      <c r="E35" s="101" t="s">
+      <c r="E35" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="F35" s="91" t="s">
+      <c r="F35" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="G35" s="107"/>
+      <c r="G35" s="102"/>
       <c r="H35" s="80" t="s">
         <v>179</v>
       </c>
-      <c r="I35" s="5"/>
+      <c r="I35" s="50"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
     </row>
     <row r="36" spans="1:13" ht="145.5" customHeight="1">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="B36" s="101" t="s">
+      <c r="B36" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="85" t="s">
+      <c r="C36" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="D36" s="111" t="s">
+      <c r="D36" s="97" t="s">
         <v>182</v>
       </c>
-      <c r="E36" s="112" t="s">
+      <c r="E36" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="F36" s="62" t="s">
+      <c r="F36" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="G36" s="4"/>
-      <c r="H36" s="62" t="s">
+      <c r="G36" s="102"/>
+      <c r="H36" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="I36" s="5"/>
+      <c r="I36" s="50"/>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
     </row>
     <row r="37" spans="1:13" ht="106.5">
-      <c r="A37" s="10" t="s">
+      <c r="A37" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="102" t="s">
         <v>187</v>
       </c>
       <c r="D37" s="80" t="s">
         <v>188</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F37" s="114" t="s">
+      <c r="F37" s="104" t="s">
         <v>189</v>
       </c>
-      <c r="G37" s="3" t="s">
+      <c r="G37" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="H37" s="113" t="s">
+      <c r="H37" s="90" t="s">
         <v>191</v>
       </c>
-      <c r="I37" s="5"/>
+      <c r="I37" s="50"/>
       <c r="J37" s="5"/>
       <c r="K37" s="5"/>
       <c r="L37" s="5"/>
       <c r="M37" s="5"/>
     </row>
     <row r="38" spans="1:13" s="1" customFormat="1" ht="137.25">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D38" s="62" t="s">
+      <c r="D38" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="E38" s="101" t="s">
+      <c r="E38" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="G38" s="3"/>
-      <c r="H38" s="62" t="s">
+      <c r="G38" s="18"/>
+      <c r="H38" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="I38" s="76">
+      <c r="I38" s="96">
         <v>46182</v>
       </c>
       <c r="J38" s="76">
@@ -3198,168 +3409,316 @@
       </c>
     </row>
     <row r="39" spans="1:13" ht="134.25" customHeight="1">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="D39" s="62" t="s">
+      <c r="D39" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="E39" s="62" t="s">
+      <c r="E39" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="F39" s="115">
+      <c r="F39" s="105">
         <v>46204</v>
       </c>
-      <c r="G39" s="4"/>
-      <c r="H39" s="109" t="s">
+      <c r="G39" s="102"/>
+      <c r="H39" s="97" t="s">
         <v>200</v>
       </c>
-      <c r="I39" s="5"/>
-      <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
-      <c r="L39" s="5"/>
-      <c r="M39" s="5"/>
-    </row>
-    <row r="40" spans="1:13">
-      <c r="A40" s="10"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="5"/>
-    </row>
-    <row r="41" spans="1:13">
-      <c r="A41" s="10"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
-      <c r="L41" s="5"/>
-      <c r="M41" s="5"/>
-    </row>
-    <row r="42" spans="1:13">
-      <c r="A42" s="10"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="5"/>
+      <c r="I39" s="111"/>
+      <c r="J39" s="85"/>
+      <c r="K39" s="85"/>
+      <c r="L39" s="85"/>
+      <c r="M39" s="85"/>
+    </row>
+    <row r="40" spans="1:13" ht="230.25" customHeight="1">
+      <c r="A40" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="H40" s="97" t="s">
+        <v>205</v>
+      </c>
+      <c r="I40" s="112"/>
+      <c r="J40" s="82"/>
+      <c r="K40" s="82"/>
+      <c r="L40" s="82"/>
+      <c r="M40" s="82"/>
+    </row>
+    <row r="41" spans="1:13" ht="71.25">
+      <c r="A41" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="D41" s="90" t="s">
+        <v>208</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F41" s="106" t="s">
+        <v>209</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H41" s="107" t="s">
+        <v>205</v>
+      </c>
+      <c r="I41" s="114"/>
+      <c r="J41" s="98"/>
+      <c r="K41" s="98"/>
+      <c r="L41" s="98"/>
+      <c r="M41" s="98"/>
+    </row>
+    <row r="42" spans="1:13" ht="66.75" customHeight="1">
+      <c r="A42" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="E42" s="102" t="s">
+        <v>213</v>
+      </c>
+      <c r="F42" s="108" t="s">
+        <v>214</v>
+      </c>
+      <c r="G42" s="102"/>
+      <c r="H42" s="109" t="s">
+        <v>215</v>
+      </c>
+      <c r="I42" s="50"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
     </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="10"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="5"/>
+    <row r="43" spans="1:13" ht="75.75">
+      <c r="A43" s="123" t="s">
+        <v>216</v>
+      </c>
+      <c r="B43" s="124" t="s">
+        <v>117</v>
+      </c>
+      <c r="C43" s="125" t="s">
+        <v>217</v>
+      </c>
+      <c r="D43" s="126" t="s">
+        <v>218</v>
+      </c>
+      <c r="E43" s="126" t="s">
+        <v>219</v>
+      </c>
+      <c r="F43" s="127" t="s">
+        <v>220</v>
+      </c>
+      <c r="G43" s="124" t="s">
+        <v>204</v>
+      </c>
+      <c r="H43" s="125"/>
+      <c r="I43" s="111"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5"/>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
     </row>
-    <row r="44" spans="1:13">
-      <c r="A44" s="10"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="5"/>
-      <c r="J44" s="5"/>
+    <row r="44" spans="1:13" ht="76.5">
+      <c r="A44" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="102" t="s">
+        <v>222</v>
+      </c>
+      <c r="D44" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="E44" s="121" t="s">
+        <v>224</v>
+      </c>
+      <c r="F44" s="122" t="s">
+        <v>225</v>
+      </c>
+      <c r="G44" s="102"/>
+      <c r="H44" s="80" t="s">
+        <v>226</v>
+      </c>
+      <c r="I44" s="82"/>
+      <c r="J44" s="50"/>
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
       <c r="M44" s="5"/>
     </row>
-    <row r="45" spans="1:13">
-      <c r="A45" s="10"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="5"/>
+    <row r="45" spans="1:13" ht="42.75" customHeight="1">
+      <c r="A45" s="93" t="s">
+        <v>227</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45" s="94" t="s">
+        <v>228</v>
+      </c>
+      <c r="D45" s="118" t="s">
+        <v>229</v>
+      </c>
+      <c r="E45" s="119" t="s">
+        <v>230</v>
+      </c>
+      <c r="F45" s="120" t="s">
+        <v>231</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H45" s="117" t="s">
+        <v>232</v>
+      </c>
+      <c r="I45" s="98"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5"/>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
     </row>
-    <row r="46" spans="1:13">
-      <c r="A46" s="10"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
+    <row r="46" spans="1:13" ht="41.25" customHeight="1">
+      <c r="A46" s="93" t="s">
+        <v>233</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46" s="94" t="s">
+        <v>234</v>
+      </c>
+      <c r="D46" s="118" t="s">
+        <v>229</v>
+      </c>
+      <c r="E46" s="119" t="s">
+        <v>230</v>
+      </c>
+      <c r="F46" s="120" t="s">
+        <v>235</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="H46" s="117" t="s">
+        <v>237</v>
+      </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
     </row>
-    <row r="47" spans="1:13">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="5"/>
-      <c r="J47" s="5"/>
-      <c r="K47" s="5"/>
-      <c r="L47" s="5"/>
-      <c r="M47" s="5"/>
-    </row>
-    <row r="48" spans="1:13">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="5"/>
+    <row r="47" spans="1:13" s="1" customFormat="1" ht="60" customHeight="1">
+      <c r="A47" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D47" s="62" t="s">
+        <v>240</v>
+      </c>
+      <c r="E47" s="119" t="s">
+        <v>230</v>
+      </c>
+      <c r="F47" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="G47" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="H47" s="62" t="s">
+        <v>241</v>
+      </c>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+    </row>
+    <row r="48" spans="1:13" s="24" customFormat="1" ht="75" customHeight="1">
+      <c r="A48" s="61" t="s">
+        <v>242</v>
+      </c>
+      <c r="B48" s="62" t="s">
+        <v>117</v>
+      </c>
+      <c r="C48" s="74" t="s">
+        <v>243</v>
+      </c>
+      <c r="D48" s="62" t="s">
+        <v>244</v>
+      </c>
+      <c r="E48" s="121" t="s">
+        <v>224</v>
+      </c>
+      <c r="F48" s="87" t="s">
+        <v>245</v>
+      </c>
+      <c r="G48" s="62" t="s">
+        <v>126</v>
+      </c>
+      <c r="H48" s="62" t="s">
+        <v>246</v>
+      </c>
+      <c r="I48" s="128">
+        <v>46218</v>
+      </c>
+      <c r="J48" s="75">
+        <v>46220</v>
+      </c>
+      <c r="K48" s="75">
+        <v>46223</v>
+      </c>
+      <c r="L48" s="75">
+        <v>46223</v>
+      </c>
+      <c r="M48" s="75">
+        <v>46223</v>
+      </c>
     </row>
     <row r="49" spans="1:13">
       <c r="A49" s="3"/>
@@ -3845,7 +4204,9 @@
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="4"/>
-      <c r="D81" s="4"/>
+      <c r="D81" s="4" t="s">
+        <v>247</v>
+      </c>
       <c r="E81" s="4"/>
       <c r="F81" s="4"/>
       <c r="G81" s="4"/>
@@ -4890,6 +5251,36 @@
       <c r="K150" s="5"/>
       <c r="L150" s="5"/>
       <c r="M150" s="5"/>
+    </row>
+    <row r="151" spans="1:13">
+      <c r="A151" s="3"/>
+      <c r="B151" s="3"/>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="4"/>
+      <c r="H151" s="4"/>
+      <c r="I151" s="5"/>
+      <c r="J151" s="5"/>
+      <c r="K151" s="5"/>
+      <c r="L151" s="5"/>
+      <c r="M151" s="5"/>
+    </row>
+    <row r="152" spans="1:13">
+      <c r="A152" s="3"/>
+      <c r="B152" s="3"/>
+      <c r="C152" s="4"/>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4"/>
+      <c r="F152" s="4"/>
+      <c r="G152" s="4"/>
+      <c r="H152" s="4"/>
+      <c r="I152" s="5"/>
+      <c r="J152" s="5"/>
+      <c r="K152" s="5"/>
+      <c r="L152" s="5"/>
+      <c r="M152" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4910,17 +5301,17 @@
   <sheetData>
     <row r="2" spans="1:8" ht="15.75">
       <c r="A2" s="65" t="s">
-        <v>201</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="20.25" customHeight="1">
       <c r="A4" s="66" t="s">
-        <v>202</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="55" customFormat="1" ht="83.25" customHeight="1">
       <c r="A5" s="64" t="s">
-        <v>203</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -4928,12 +5319,12 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="66" t="s">
-        <v>204</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="84" customHeight="1">
       <c r="A8" s="64" t="s">
-        <v>205</v>
+        <v>252</v>
       </c>
       <c r="H8" s="56"/>
     </row>

</xml_diff>